<commit_message>
Remove duplicate prompt log file
</commit_message>
<xml_diff>
--- a/Excel/Test Cases _Checklist _Test Summary Report.xlsx
+++ b/Excel/Test Cases _Checklist _Test Summary Report.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30524"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="804" documentId="11_92480E3D80EBD8D2623DC6FA873E8C18510380D4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BE62EE4-1085-413A-8E49-F7BB1FD75B02}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{06832F97-62AC-44D8-BD2D-7B6604538728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST_CASE" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="115">
   <si>
     <t>TC ID </t>
   </si>
@@ -372,6 +372,16 @@
   </si>
   <si>
     <t>Video</t>
+  </si>
+  <si>
+    <t>TC in Video</t>
+  </si>
+  <si>
+    <t>TC01
+TC02
+TC03
+TC04
+TC05</t>
   </si>
   <si>
     <t>Requirement</t>
@@ -518,7 +528,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -605,6 +615,14 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -654,7 +672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -730,13 +748,14 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1473,34 +1492,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8B4E4C7-4312-4387-9BCE-4BC508A03251}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="25.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:2" ht="15.75">
+      <c r="A1" s="31" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="31" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="B2" s="30">
+      <c r="B2" s="29">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="30">
+      <c r="B3" s="29">
         <v>3</v>
       </c>
     </row>
@@ -1529,11 +1548,19 @@
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="30">
         <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="76.5">
+      <c r="A8" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1552,63 +1579,63 @@
   <sheetData>
     <row r="1" spans="1:2" ht="21">
       <c r="A1" s="13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="129">
       <c r="A2" s="20" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="96.75">
       <c r="A3" s="16" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="113.25">
       <c r="A4" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" s="21" t="s">
         <v>100</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="81">
       <c r="A5" s="22" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="91.5">
       <c r="A6" s="26" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="60.75">
       <c r="A7" s="15" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="40.5" customHeight="1">
       <c r="A8" s="15" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B8" s="19" t="s">
         <v>76</v>
@@ -1616,66 +1643,66 @@
     </row>
     <row r="9" spans="1:2" ht="60.75">
       <c r="A9" s="23" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18.75">
       <c r="A10" s="24" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="45.75">
       <c r="A11" s="23" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="60.75">
       <c r="A12" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="24.75" customHeight="1">
       <c r="A13" s="25" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24.75" customHeight="1">
       <c r="A14" s="25" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="45.75">
       <c r="A15" s="27" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="45.75">
       <c r="A16" s="23" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>